<commit_message>
Add phone normalization, deduplication, and .review quarantine
- Strip non-digits; handle 0057 prefix
- 10-digit numbers starting with 3 get 57 prepended
- Valid 12-digit 573 numbers pass through unchanged
- Duplicates and invalid numbers routed to .review files
- Output files now contain only clean, unique, normalized numbers
</commit_message>
<xml_diff>
--- a/output/campaign_Vive_Living.xlsx
+++ b/output/campaign_Vive_Living.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C322"/>
+  <dimension ref="A1:C321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5774,117 +5774,100 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>573043460864</t>
+          <t>573124457430</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Laura Martinez</t>
+          <t>Juan Or.mm</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>60539594514</t>
+          <t>59570787255</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>573124457430</t>
+          <t>573127938080</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Juan Or.mm</t>
+          <t>Monica De La Hoz</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>59570787255</t>
+          <t>60074896916</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>573127938080</t>
+          <t>573187620912</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Monica De La Hoz</t>
+          <t>Cielo Rios</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>60074896916</t>
+          <t>60676243800</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>573187620912</t>
+          <t>573205309193</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Cielo Rios</t>
+          <t>Álvaro Fernando Portilla Araujo</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>60676243800</t>
+          <t>60139210154</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>573205309193</t>
+          <t>573006545177</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Álvaro Fernando Portilla Araujo</t>
+          <t>Daniel Arango</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>60139210154</t>
+          <t>59332807266</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>573006545177</t>
+          <t>573116204753</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Daniel Arango</t>
+          <t>Juanjose Galvis González</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
-        <is>
-          <t>59332807266</t>
-        </is>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="inlineStr">
-        <is>
-          <t>573116204753</t>
-        </is>
-      </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>Juanjose Galvis González</t>
-        </is>
-      </c>
-      <c r="C322" t="inlineStr">
         <is>
           <t>59247487496</t>
         </is>

</xml_diff>